<commit_message>
implement p1 perf opt plan
</commit_message>
<xml_diff>
--- a/wiki/development-plan/performance-optimization-plan.xlsx
+++ b/wiki/development-plan/performance-optimization-plan.xlsx
@@ -815,12 +815,12 @@
     <row r="20">
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>P1 — Ref-data hoist</t>
+          <t>P1 — Ref-data hoist  ✅ 4/4</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Accounts/categories fetched once via a context provider, not per page mount.  •  Frontend</t>
+          <t>DONE &amp; VERIFIED live: FinanceDataProvider in the ROOT layout fetches accounts + categories once per session; client-side navigation no longer re-fetches reference data. See p1-implementation-note.md.  •  Frontend</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="K10" s="19" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="K11" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="K12" s="19" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
implement p2 perf opt plan
</commit_message>
<xml_diff>
--- a/wiki/development-plan/performance-optimization-plan.xlsx
+++ b/wiki/development-plan/performance-optimization-plan.xlsx
@@ -827,12 +827,12 @@
     <row r="21">
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>P2 — Cache hardening</t>
+          <t>P2 — Cache hardening  ✅ 3/3</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Per-collection TTL; single-resource refresh instead of all-or-nothing.  •  Backend</t>
+          <t>DONE &amp; unit-verified: per-collection TTL freshness (LIVE_CACHE_TTL_MS, default 45s) + per-resource loaders. Cold start = 5 queries; warm read = 0; stale = 1 (that collection only). See p2-implementation-note.md.  •  Backend</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="K14" s="19" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
implement p3 perf opt plan
</commit_message>
<xml_diff>
--- a/wiki/development-plan/performance-optimization-plan.xlsx
+++ b/wiki/development-plan/performance-optimization-plan.xlsx
@@ -839,12 +839,12 @@
     <row r="22">
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>P3 — React Query</t>
+          <t>P3 — React Query  ◑ 5/6</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Durable caching, dedup, optimistic mutations, background refetch.  •  Frontend (ADR by Architect)</t>
+          <t>DONE: ADR, RQ provider, reads on useQuery (useApiData removed), cross-section invalidation. Also found+fixed a P2-introduced cold-load thundering-herd bug (single-flight). P3-6 final clean CRUD regression pending Notion rate-limit recovery. See p3-implementation-note.md + adr-001.  •  Frontend</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="K18" s="19" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="K20" s="19" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="K22" s="19" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
impl p4 opt plan, not yet done
</commit_message>
<xml_diff>
--- a/wiki/development-plan/performance-optimization-plan.xlsx
+++ b/wiki/development-plan/performance-optimization-plan.xlsx
@@ -851,12 +851,12 @@
     <row r="23">
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>P4 — Refactor</t>
+          <t>P4 — Refactor  ◔ in progress</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Split workspace monolith + NotionService god class behind stable contracts.  •  Frontend + Backend</t>
+          <t>Boundary plan DONE. Bottom-up extractions landed &amp; verified: FE lib/finance-helpers + finance-events; BE notion-resource-utils + LiveCacheManager (NotionService 1138-&gt;827 lines, cache spec 6/6 green). Remaining page/service splits sequenced.  •  Frontend + Backend</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="K24" s="19" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
     </row>

</xml_diff>